<commit_message>
Refactor code structure and remove redundant code blocks for improved readability and maintainability
</commit_message>
<xml_diff>
--- a/src/assets/files/catalog.xlsx
+++ b/src/assets/files/catalog.xlsx
@@ -1002,10 +1002,10 @@
         <v>MULTI-FAMILY</v>
       </c>
       <c r="H21" t="str">
-        <v/>
+        <v>08-Pictures/GRIFFIN</v>
       </c>
       <c r="I21" t="str">
-        <v/>
+        <v>01-PRINCIPAL-new.webp</v>
       </c>
     </row>
     <row r="22">
@@ -1060,10 +1060,10 @@
         <v>COMMERCIAL</v>
       </c>
       <c r="H23" t="str">
-        <v/>
+        <v>08-Pictures/MALL 163</v>
       </c>
       <c r="I23" t="str">
-        <v/>
+        <v>01.webp</v>
       </c>
     </row>
     <row r="24">
@@ -1089,10 +1089,10 @@
         <v>MULTI-FAMILY</v>
       </c>
       <c r="H24" t="str">
-        <v/>
+        <v>08-Pictures/LUX GROVE</v>
       </c>
       <c r="I24" t="str">
-        <v/>
+        <v>01-PRINCIPAL.webp</v>
       </c>
     </row>
     <row r="25">
@@ -1167,7 +1167,7 @@
         <v>LLR ARCHITECTS,INC</v>
       </c>
       <c r="E27" t="str">
-        <v/>
+        <v>Structural design engineering services for 10 units multi-family development. Including a concrete structure with a precast joist and a concrete shear wall.</v>
       </c>
       <c r="F27" t="str">
         <v>Hollywood, FL</v>
@@ -1196,7 +1196,7 @@
         <v>WHA Design</v>
       </c>
       <c r="E28" t="str">
-        <v/>
+        <v>Structural design engineering services for renovating and adding to the existing church, including new educational spaces and multipurpose rooms, in combination with a steel and masonry structure with metal joists and a concrete roof.</v>
       </c>
       <c r="F28" t="str">
         <v>Miami, FL</v>

</xml_diff>